<commit_message>
Add osi-email-sender skill, hard-rule CLAUDE.md, 4pm send log, scheduled tasks v2
</commit_message>
<xml_diff>
--- a/prospects-tracker-new.xlsx
+++ b/prospects-tracker-new.xlsx
@@ -20,8 +20,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -95,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -111,6 +112,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -476,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I330"/>
+  <dimension ref="A1:I335"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -15722,7 +15724,6 @@
           <t>SiFi Networks</t>
         </is>
       </c>
-      <c r="D328" t="inlineStr"/>
       <c r="E328" t="inlineStr">
         <is>
           <t>SmartOptics transceivers (primary), DWDM backbone (secondary)</t>
@@ -15834,6 +15835,231 @@
       <c r="I330" t="inlineStr">
         <is>
           <t>Dir Engineering, Verizon transmission background. Hunter just closed Oak Hill Capital deal for Oregon expansion. Optics lead. Day 1 2026-05-07. Person 6 at Hunter (+10 biz day cooling gap).</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>Paul Merritt</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>Chief Executive Officer</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>Fatbeam</t>
+        </is>
+      </c>
+      <c r="D331" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/pamerritt/</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>Exec supply chain / DWDM / TPM</t>
+        </is>
+      </c>
+      <c r="F331" t="inlineStr">
+        <is>
+          <t>Andy -- HubSpot ID 216986522272</t>
+        </is>
+      </c>
+      <c r="G331" t="inlineStr">
+        <is>
+          <t>Pursue -- sequence live</t>
+        </is>
+      </c>
+      <c r="H331" s="9" t="n">
+        <v>46133</v>
+      </c>
+      <c r="I331" t="inlineStr">
+        <is>
+          <t>CEO, 2nd degree. Hook: 1mo-old post about Western WA Enterprise team hiring during Basalt buildout. Exec angle, not sample opener.</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>Gavin Budd</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>VP of Network Operations and Engineering</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>Fatbeam</t>
+        </is>
+      </c>
+      <c r="D332" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/gavin-budd-99a7253/</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>DWDM / Optics (SFP sample wedge) / TPM</t>
+        </is>
+      </c>
+      <c r="F332" t="inlineStr">
+        <is>
+          <t>Andy -- HubSpot ID 538744</t>
+        </is>
+      </c>
+      <c r="G332" t="inlineStr">
+        <is>
+          <t>Pursue -- sequence live</t>
+        </is>
+      </c>
+      <c r="H332" s="9" t="n">
+        <v>46133</v>
+      </c>
+      <c r="I332" t="inlineStr">
+        <is>
+          <t>VP Network Ops, 2nd degree, restricted profile. Existing HubSpot contact (last touch Aug 2020). Lead SFP sample then DWDM vs Ciena/Nokia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>Danny Pate</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>Chief Operating Officer</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>Fatbeam</t>
+        </is>
+      </c>
+      <c r="D333" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/dannypate/</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>TPM / DWDM / Pre-owned networking (COO exec angle)</t>
+        </is>
+      </c>
+      <c r="F333" t="inlineStr">
+        <is>
+          <t>Andy -- HubSpot ID 216990632756</t>
+        </is>
+      </c>
+      <c r="G333" t="inlineStr">
+        <is>
+          <t>Pursue -- sequence live</t>
+        </is>
+      </c>
+      <c r="H333" s="9" t="n">
+        <v>46133</v>
+      </c>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>COO, 3rd degree, active on LinkedIn. Lead TPM / OEM cost conversation. Fatbeam PE-backed expansion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>Adam Hill</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>NOC Manager</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>Fatbeam</t>
+        </is>
+      </c>
+      <c r="D334" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/adam-hill-b31136229/</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>SFP break-glass / TPM / Pre-owned networking</t>
+        </is>
+      </c>
+      <c r="F334" t="inlineStr">
+        <is>
+          <t>Andy -- HubSpot ID 216990215766</t>
+        </is>
+      </c>
+      <c r="G334" t="inlineStr">
+        <is>
+          <t>Pursue -- sequence live</t>
+        </is>
+      </c>
+      <c r="H334" s="9" t="n">
+        <v>46133</v>
+      </c>
+      <c r="I334" t="inlineStr">
+        <is>
+          <t>NOC Manager, 3rd degree. Lead SFP break-glass for 2am failures then TPM on aging gear.</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>Jordan Diaz</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>OSP Engineering Manager (ZI: Manager Network Operations)</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>Fatbeam</t>
+        </is>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/jordan-diaz-095b73184/</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>DWDM / Optics / 400G ZR</t>
+        </is>
+      </c>
+      <c r="F335" t="inlineStr">
+        <is>
+          <t>Andy -- HubSpot ID 216979127691</t>
+        </is>
+      </c>
+      <c r="G335" t="inlineStr">
+        <is>
+          <t>Pursue -- sequence live</t>
+        </is>
+      </c>
+      <c r="H335" s="9" t="n">
+        <v>46133</v>
+      </c>
+      <c r="I335" t="inlineStr">
+        <is>
+          <t>OSP Eng Mgr / dual Network Ops Mgr per ZoomInfo. 3rd degree. Lead SFP sample then DWDM for transport buildout.</t>
         </is>
       </c>
     </row>
@@ -15849,7 +16075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -17298,6 +17524,36 @@
       <c r="F50" t="inlineStr">
         <is>
           <t>18 emails queued to email-queue.json. LINKED_IN_CONNECT tasks 107848632473 (David), 107882380691 (Ed), 107849563414 (Joseph) marked COMPLETED. New Day-1 LinkedIn tasks created: 108266943518 (David, due 2026-04-21), 108276392767 (Ed, due 2026-04-21), 108275895457 (Joseph, due 2026-05-07). Weekend scheduled batch 27 of 38. Strategy notes already in place from 2026-04-11 qualification run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Fatbeam</t>
+        </is>
+      </c>
+      <c r="B51" s="9" t="n">
+        <v>46133</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>19 qualified shortlist reviewed, 5 sequenced</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>5 sequences (Paul Merritt CEO, Gavin Budd VP Net Ops, Danny Pate COO, Adam Hill NOC Mgr, Jordan Diaz OSP/Net Ops)</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Basalt Infrastructure acquiring from SDC Capital closing Q2 2026. Fatbeam owned by Andy, last contacted Aug 2020. Cold reengagement. Approved-vendor status: No. Also flagged: Gregory Green (HubSpot 355102) is former CEO, no longer at Fatbeam; contact record needs update. Katherine Stephens, Jeffrey Bulger disqualified on profile read (BI/GIS and Open To Work respectively). 6 other individual contributor engineers/NOC not sequenced (too junior for full 6-email).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
End of day: skills cleanup, osi-email-sender skill, scheduled tasks v2, zip snapshot
</commit_message>
<xml_diff>
--- a/prospects-tracker-new.xlsx
+++ b/prospects-tracker-new.xlsx
@@ -17568,7 +17568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -17659,6 +17659,39 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Gary Duttenhefer</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Consolidated Telcom</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Hard bounce -- bad email address</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" t="n">
+        <v>4</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>garyduttenhefer@consolidatednd.com bounced 4/22 after email 2/6. HubSpot also shows garyduttenhefer48645152@gmail.com on record. HubSpot note added.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
queue path back to Claude-Brain + skill rewrites + overnight state + new hard rules
</commit_message>
<xml_diff>
--- a/prospects-tracker-new.xlsx
+++ b/prospects-tracker-new.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I335"/>
+  <dimension ref="A1:I338"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -16060,6 +16060,141 @@
       <c r="I335" t="inlineStr">
         <is>
           <t>OSP Eng Mgr / dual Network Ops Mgr per ZoomInfo. 3rd degree. Lead SFP sample then DWDM for transport buildout.</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>Jesse Tucker</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>Network Engineer IV (DOCSIS)</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>Midcontinent Communications, Inc.</t>
+        </is>
+      </c>
+      <c r="D336" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/jesse-tucker6128/</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>Sample SFPs (Network) -&gt; DWDM (cable transport) -&gt; Cisco TPM -&gt; DIMMs</t>
+        </is>
+      </c>
+      <c r="F336" t="inlineStr">
+        <is>
+          <t>Andy -- HubSpot ID 217781724059</t>
+        </is>
+      </c>
+      <c r="G336" t="inlineStr">
+        <is>
+          <t>Pursue -- sequence live</t>
+        </is>
+      </c>
+      <c r="H336" s="8" t="n">
+        <v>46137</v>
+      </c>
+      <c r="I336" t="inlineStr">
+        <is>
+          <t>Network Eng IV DOCSIS at Midco. Wireshark Cert Analyst 1mo, DOCSIS Eng Pro, Cisco CCNP-Enterprise. SCI Broadband acquisition adding plant. Day 1 = 2026-05-28 (5th Midco person, +10 bd cooling gap).</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>Tony Fisher</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>System Engineer</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>Midcontinent Communications, Inc.</t>
+        </is>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/tony-fisher-a270506/</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>DIMMs (Server) -&gt; Sample SFPs -&gt; Cisco TPM -&gt; DWDM</t>
+        </is>
+      </c>
+      <c r="F337" t="inlineStr">
+        <is>
+          <t>Andy -- HubSpot ID 564828</t>
+        </is>
+      </c>
+      <c r="G337" t="inlineStr">
+        <is>
+          <t>Pursue -- sequence live</t>
+        </is>
+      </c>
+      <c r="H337" s="8" t="n">
+        <v>46137</v>
+      </c>
+      <c r="I337" t="inlineStr">
+        <is>
+          <t>System Engineer at Midco, 30-39 yrs exp, IT Infrastructure. HubSpot updated: jobtitle stale, phone/mobile re-keyed off switchboard. Day 1 = 2026-06-03 (6th Midco, +4 bd).</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>Brad Janzen</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Transport Engineering Supervisor</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Midcontinent Communications, Inc.</t>
+        </is>
+      </c>
+      <c r="D338" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/brad-janzen-3302917/</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>DWDM (pain-led) -&gt; Sample SFPs -&gt; Cisco TPM -&gt; DIMMs</t>
+        </is>
+      </c>
+      <c r="F338" t="inlineStr">
+        <is>
+          <t>Andy -- HubSpot ID 217780773512</t>
+        </is>
+      </c>
+      <c r="G338" t="inlineStr">
+        <is>
+          <t>Pursue -- sequence live</t>
+        </is>
+      </c>
+      <c r="H338" s="8" t="n">
+        <v>46137</v>
+      </c>
+      <c r="I338" t="inlineStr">
+        <is>
+          <t>Transport Engineering Supervisor at Midco, 30+ yrs, Manager. Direct DWDM buyer. SCI Broadband hook. Day 1 = 2026-06-09 (7th Midco, +4 bd).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
saturday overnight + daytime — 16 sequences fired, 101 pending
</commit_message>
<xml_diff>
--- a/prospects-tracker-new.xlsx
+++ b/prospects-tracker-new.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I338"/>
+  <dimension ref="A1:I347"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -16195,6 +16195,417 @@
       <c r="I338" t="inlineStr">
         <is>
           <t>Transport Engineering Supervisor at Midco, 30+ yrs, Manager. Direct DWDM buyer. SCI Broadband hook. Day 1 = 2026-06-09 (7th Midco, +4 bd).</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>John Lachance</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Sr. Solutions Engineer</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>Lingo Communications</t>
+        </is>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/jlachance/</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>Sample SFPs (Network) -&gt; Cisco/Juniper TPM -&gt; DWDM (Smartoptics) -&gt; DIMMs</t>
+        </is>
+      </c>
+      <c r="F339" t="inlineStr">
+        <is>
+          <t>Andy -- HubSpot ID 217783919683</t>
+        </is>
+      </c>
+      <c r="G339" t="inlineStr">
+        <is>
+          <t>Pursue -- sequence live</t>
+        </is>
+      </c>
+      <c r="H339" s="8" t="n">
+        <v>46137</v>
+      </c>
+      <c r="I339" t="inlineStr">
+        <is>
+          <t>Sr Solutions Engineer at Lingo (3rd-degree). ZoomInfo FULL_MATCH 98%: jlachance@impacttelecom.com (legacy Lingo brand domain) + mobile (512) 635-1720. Network sample-offer w/ TPM/DWDM/DIMMs follow-on. Day 1 = 2026-04-27 (1st Lingo, person_count=0 -&gt; next bd).</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>Colin Vesper</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>Lead Network Engineer</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>Visionary Broadband</t>
+        </is>
+      </c>
+      <c r="D340" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/colinvesper/</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>Sample SFPs (Network) -&gt; DWDM (Smartoptics) -&gt; Cisco/Juniper TPM -&gt; DIMMs</t>
+        </is>
+      </c>
+      <c r="F340" t="inlineStr">
+        <is>
+          <t>Andy -- HubSpot ID 217774992137</t>
+        </is>
+      </c>
+      <c r="G340" t="inlineStr">
+        <is>
+          <t>Pursue -- sequence live</t>
+        </is>
+      </c>
+      <c r="H340" s="8" t="n">
+        <v>46137</v>
+      </c>
+      <c r="I340" t="inlineStr">
+        <is>
+          <t>Lead Network Engineer at Visionary Broadband (3rd-degree, Gillette WY). ZoomInfo 93%: cvesper@office.vcn.com + (307) 685-5523 direct + (307) 680-7624 mobile. Visionary is existing OSI customer at company level. Day 1 = 2026-04-27 (1st Visionary).</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>Preston Schilling</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>COO</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>Visionary Broadband</t>
+        </is>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/preston-schilling-48921626/</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>DWDM (pain-led, exec) -&gt; TPM -&gt; DIMMs -&gt; Pre owned + new networking</t>
+        </is>
+      </c>
+      <c r="F341" t="inlineStr">
+        <is>
+          <t>Andy -- HubSpot ID 217794530995</t>
+        </is>
+      </c>
+      <c r="G341" t="inlineStr">
+        <is>
+          <t>Pursue -- sequence live</t>
+        </is>
+      </c>
+      <c r="H341" s="8" t="n">
+        <v>46137</v>
+      </c>
+      <c r="I341" t="inlineStr">
+        <is>
+          <t>COO at Visionary Broadband (1st-degree, Gillette WY). ZoomInfo 98%: pschilling@office.vcn.com + (307) 685-5545 direct + (307) 689-3416 mobile. Already 1st-degree, LINKED_IN_CONNECT skipped. Pain-led DWDM exec opener. Day 1 = 2026-05-01 (2nd Visionary, +4 bd from Colin).</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>Sarah Frisbie</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Director, Network Engineering</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>altafiber (Cincinnati Bell)</t>
+        </is>
+      </c>
+      <c r="D342" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/sarahfrisbie1/</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>Network sample SFPs -&gt; DWDM/transport (2027 fiber push) -&gt; TPM -&gt; DIMMs</t>
+        </is>
+      </c>
+      <c r="F342" t="inlineStr">
+        <is>
+          <t>Andy -- HubSpot ID 46214249386 (existing, last contact 2024-08)</t>
+        </is>
+      </c>
+      <c r="G342" t="inlineStr">
+        <is>
+          <t>Pursue -- sequence live</t>
+        </is>
+      </c>
+      <c r="H342" s="8" t="n">
+        <v>46137</v>
+      </c>
+      <c r="I342" t="inlineStr">
+        <is>
+          <t>Director Network Engineering at altafiber. 1st-degree, 2 mutual. ZoomInfo 99 percent: sarah.frisbie@altafiber.com + (513) 565-0650 mobile. Existing HubSpot mobile (513) 314-6657. Day 1 = 2026-05-11 (Cincinnati Bell run-stagger person_count=1). Hook: altafiber publicly committed to 90 percent fiber availability by 2027. 5 other altafiber sequences in flight from Andy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>Scott Pennington</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>Network Engineer III / Principal Platform Engineer</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>altafiber (Cincinnati Bell)</t>
+        </is>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/scott-pennington-3b0670b/</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>Network sample SFPs -&gt; DWDM/transport (2027 fiber) -&gt; TPM -&gt; DIMMs</t>
+        </is>
+      </c>
+      <c r="F343" t="inlineStr">
+        <is>
+          <t>Andy -- HubSpot ID 138771300470 (existing, last contact 2025-10-10)</t>
+        </is>
+      </c>
+      <c r="G343" t="inlineStr">
+        <is>
+          <t>Pursue -- sequence live (re-engagement)</t>
+        </is>
+      </c>
+      <c r="H343" s="8" t="n">
+        <v>46137</v>
+      </c>
+      <c r="I343" t="inlineStr">
+        <is>
+          <t>Senior IC at altafiber. LinkedIn says Network Engineer III, HubSpot+ZoomInfo say Principal Platform Engineer (more recent). 1st-degree (3 mutuals). ZoomInfo 91 percent: scott.pennington@altafiber.com. Day 1 = 2026-05-15. Sister sequence to Sarah Frisbie (Director, 5/11).</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>Ron Beerman</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>Chief Network Officer</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>altafiber (Cincinnati Bell)</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/ron-beerman-a4407a2/</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>DWDM/transport pain-led exec -&gt; TPM -&gt; DIMMs -&gt; Pre owned + new Nokia</t>
+        </is>
+      </c>
+      <c r="F344" t="inlineStr">
+        <is>
+          <t>Andy -- HubSpot ID 3732051 (existing since 2024-02, long re-engagement)</t>
+        </is>
+      </c>
+      <c r="G344" t="inlineStr">
+        <is>
+          <t>Pursue -- sequence live (exec, pain-led)</t>
+        </is>
+      </c>
+      <c r="H344" s="8" t="n">
+        <v>46137</v>
+      </c>
+      <c r="I344" t="inlineStr">
+        <is>
+          <t>CNO at altafiber. 1st-degree, 1 mutual (Todd). ZoomInfo 99 percent: ron.beerman@altafiber.com + mobile (513) 608-7400. Hook: Lahaina restoration talk at FiberConnect 2025 + altafiber 90 percent fiber by 2027 commitment. Pain-led exec opener (SmartOptics DCP DWDM vs Ciena/Nokia, 30-50 percent below). Day 1 = 2026-05-21. Sister sequences: Frisbie (5/11), Pennington (5/15).</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>Stephen Linde</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>Director, Procurement</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>altafiber</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/steve-linde-20403140/</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>Pain-led DWDM/transport intro to Procurement Director, expand to TPM + DIMMs + pre-owned across the sequence</t>
+        </is>
+      </c>
+      <c r="F345" t="inlineStr">
+        <is>
+          <t>Andy</t>
+        </is>
+      </c>
+      <c r="G345" t="inlineStr">
+        <is>
+          <t>Pursue</t>
+        </is>
+      </c>
+      <c r="H345" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="I345" t="inlineStr">
+        <is>
+          <t>1st degree, LINKED_IN_CONNECT skipped. Day 1 2026-05-28. Cincinnati Bell stagger person 4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>Justin Pastore</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>Senior Network and Security Engineer</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>Armstrong Group of Companies</t>
+        </is>
+      </c>
+      <c r="D346" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/justin-pastore-39b79880/</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>Network sample-offer (free SFP), pivot to DWDM, TPM, DIMMs, and pre-owned gear</t>
+        </is>
+      </c>
+      <c r="F346" t="inlineStr">
+        <is>
+          <t>Andy</t>
+        </is>
+      </c>
+      <c r="G346" t="inlineStr">
+        <is>
+          <t>Pursue</t>
+        </is>
+      </c>
+      <c r="H346" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="I346" t="inlineStr">
+        <is>
+          <t>Existing HubSpot 539547. Day 1 2026-04-27 (Mon). 3rd-degree LinkedIn. Cisco Networking Academy. 10+ years tenure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>Shawn Hillard</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>Manager, Network Operations</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>Armstrong Group of Companies</t>
+        </is>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/shawn-hillard-21509a37/</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>Network sample-offer (free SFP), pivot DWDM, TPM, DIMMs, pre-owned Cisco</t>
+        </is>
+      </c>
+      <c r="F347" t="inlineStr">
+        <is>
+          <t>Andy</t>
+        </is>
+      </c>
+      <c r="G347" t="inlineStr">
+        <is>
+          <t>Pursue</t>
+        </is>
+      </c>
+      <c r="H347" t="inlineStr">
+        <is>
+          <t>2026-04-25</t>
+        </is>
+      </c>
+      <c r="I347" t="inlineStr">
+        <is>
+          <t>Existing HubSpot 539438. Day 1 2026-05-01. 3rd-degree LI. NOC manager 20 years tenure since 2006.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
skill edits + prospecting system v3: stagger fix, WHO OWNS WHAT cleanup, RULES trimmed, qual/outreach boundary hardened, 5-skill package rebuilt
</commit_message>
<xml_diff>
--- a/prospects-tracker-new.xlsx
+++ b/prospects-tracker-new.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prospects" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Company Status" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unenrolled" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Companies Prospected" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospects'!$A$1:$I$1</definedName>
@@ -24,7 +25,7 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -55,8 +56,18 @@
       <name val="Arial"/>
       <color rgb="00444444"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -83,8 +94,18 @@
         <fgColor rgb="00833C00"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBF3FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -92,11 +113,25 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -113,6 +148,21 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -478,7 +528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I400"/>
+  <dimension ref="A1:I405"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -19022,6 +19072,241 @@
       <c r="I400" t="inlineStr">
         <is>
           <t>4yr in role / 30+yr exp; core IP focus, 400G transport angle; HS 140606145562</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>Mason Moesch</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>Infrastructure Engineering Manager</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>Nsight</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/masonmoesch/</t>
+        </is>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>Pain-Led TPM (NetApp)</t>
+        </is>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t>Contact exists (ID 102931114785)</t>
+        </is>
+      </c>
+      <c r="G401" t="inlineStr">
+        <is>
+          <t>6-email sequence queued, Email 1: 2026-05-04</t>
+        </is>
+      </c>
+      <c r="H401" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="I401" t="inlineStr">
+        <is>
+          <t>Promoted Feb 2026, follows NetApp on LinkedIn, Backup Solutions skill. ZI FULL_MATCH. Regional carrier WI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>Peter Whiteside</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>Vice President of Infrastructure</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>Brivo</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/peter-whiteside-1b490311/</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>TPM/multi-vendor maintenance (merger hook)</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>New contact created (ID 219246525852)</t>
+        </is>
+      </c>
+      <c r="G402" t="inlineStr">
+        <is>
+          <t>6-email sequence queued, Email 1: 2026-05-04</t>
+        </is>
+      </c>
+      <c r="H402" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="I402" t="inlineStr">
+        <is>
+          <t>Eagle Eye + Brivo merger Dec 2025. Inherited two infra stacks. ZI COMPANY_ONLY_MATCH; email pattern-inferred from brivo.com confirmed contacts. LinkedIn Path A verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>Mitch Vieu</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>Senior Manager Telecom Engineering and Operations</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>Copper Valley Telephone Cooperative</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/mitch-vieu-b785a810b/</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>Pain-Led DWDM: rural Alaska carrier, OSP + network engineering, budget owner. TPM, Pre-Owned, Optics follow-ups.</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>In sequence</t>
+        </is>
+      </c>
+      <c r="G403" t="inlineStr">
+        <is>
+          <t>6-email Pain-Led DWDM sequence queued. Day 1: 2026-05-04.</t>
+        </is>
+      </c>
+      <c r="H403" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="I403" t="inlineStr">
+        <is>
+          <t>Prior OSI engagement Oct 2023. Last contact 2.5 yrs cold. HubSpot ID 2844251.</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>Robert Geraghty</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>Lead Network Engineer</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>Copper Valley Telephone Cooperative</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>linkedin.com/in/robert-geraghty-b72b9b19b/</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>Sample-Offer Network: optical specialist running 400G DWDM/EDFA at CVTC. Secondary: DWDM supply chain, TPM, Pre-Owned.</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>In sequence</t>
+        </is>
+      </c>
+      <c r="G404" t="inlineStr">
+        <is>
+          <t>6-email Sample-Offer Network sequence queued. Day 1: 2026-05-08.</t>
+        </is>
+      </c>
+      <c r="H404" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="I404" t="inlineStr">
+        <is>
+          <t>Certified Optical Network Engineer cert Sep 2025. Built CVTC ISP (ASN:20259). Prior OSI LI contact Jan 2024. HubSpot ID 127508779633.</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>Tim Chin</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>Director of IT &amp; Security</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>Rajant Corp</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/tim-chin-rajant/</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>TPM (SmartNet savings, Cisco support), DIMMs/compute, spare optics for field nodes</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G405" t="inlineStr">
+        <is>
+          <t>6-email sequence queued (Pain-Led TPM). LinkedIn connect due 2026-05-05.</t>
+        </is>
+      </c>
+      <c r="H405" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="I405" t="inlineStr">
+        <is>
+          <t>DoD contractor, Breadcrumb mesh nodes. Cost-reduction focus (27% savings on profile). Park Place/SE merger angle for E2.</t>
         </is>
       </c>
     </row>
@@ -20657,4 +20942,1230 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C71"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="25" customHeight="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B1" s="10" t="inlineStr">
+        <is>
+          <t>Last Sequence Date</t>
+        </is>
+      </c>
+      <c r="C1" s="10" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>Midco</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>Vero Networks</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C3" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="11" t="inlineStr">
+        <is>
+          <t>Hunter Communications</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-24</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>S&amp;P Global</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>Consumer Cellular</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>Resound Networks</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>Midcontinent Communications, Inc.</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>Rackspace</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>Momentum Telecom</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>Armstrong Group of Companies</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>Fidelity Communications</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>altafiber</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>Saddleback Communications</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>Bank of America</t>
+        </is>
+      </c>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>Cantor Fitzgerald</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-18</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>Fatbeam</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>OEC Fiber</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>Patrick Industries</t>
+        </is>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>Axcent Networks</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>Copper Valley Telephone Cooperative</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="C21" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>BNY Mellon</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>Lingo Communications</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>360 Broadband</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="13" t="inlineStr">
+        <is>
+          <t>Princeton University</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="C25" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>Rajant</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>Armstrong Group</t>
+        </is>
+      </c>
+      <c r="B27" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>Altafiber</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>North American Interconnect</t>
+        </is>
+      </c>
+      <c r="B29" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="C29" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>Nsight</t>
+        </is>
+      </c>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>Consolidated Telcom</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>Desjardins</t>
+        </is>
+      </c>
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>Visionary Broadband</t>
+        </is>
+      </c>
+      <c r="B33" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="C33" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t>Brivo</t>
+        </is>
+      </c>
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>Stellar Broadband</t>
+        </is>
+      </c>
+      <c r="B35" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="C35" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t>Grande Communications</t>
+        </is>
+      </c>
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C36" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="13" t="inlineStr">
+        <is>
+          <t>Thor Industries</t>
+        </is>
+      </c>
+      <c r="B37" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C37" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t>Bergen New Bridge Medical Center</t>
+        </is>
+      </c>
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C38" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="13" t="inlineStr">
+        <is>
+          <t>SBA Communications</t>
+        </is>
+      </c>
+      <c r="B39" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C39" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="11" t="inlineStr">
+        <is>
+          <t>DFA Milk</t>
+        </is>
+      </c>
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C40" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="13" t="inlineStr">
+        <is>
+          <t>Transaction Network Services</t>
+        </is>
+      </c>
+      <c r="B41" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C41" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="11" t="inlineStr">
+        <is>
+          <t>Atlantic Health Systems</t>
+        </is>
+      </c>
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C42" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="13" t="inlineStr">
+        <is>
+          <t>Global Cloud Xchange</t>
+        </is>
+      </c>
+      <c r="B43" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C43" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="11" t="inlineStr">
+        <is>
+          <t>Baxter International</t>
+        </is>
+      </c>
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C44" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="13" t="inlineStr">
+        <is>
+          <t>WSP</t>
+        </is>
+      </c>
+      <c r="B45" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="C45" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="11" t="inlineStr">
+        <is>
+          <t>Winnebago Industries</t>
+        </is>
+      </c>
+      <c r="B46" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C46" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="13" t="inlineStr">
+        <is>
+          <t>Skywire Networks</t>
+        </is>
+      </c>
+      <c r="B47" s="14" t="inlineStr">
+        <is>
+          <t>2026-05-29</t>
+        </is>
+      </c>
+      <c r="C47" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="11" t="inlineStr">
+        <is>
+          <t>Spectrotel</t>
+        </is>
+      </c>
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="C48" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="18" customHeight="1">
+      <c r="A49" s="13" t="inlineStr">
+        <is>
+          <t>VTX1 Companies</t>
+        </is>
+      </c>
+      <c r="B49" s="14" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="C49" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="11" t="inlineStr">
+        <is>
+          <t>Docomo Pacific</t>
+        </is>
+      </c>
+      <c r="B50" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="C50" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="13" t="inlineStr">
+        <is>
+          <t>LG CNS</t>
+        </is>
+      </c>
+      <c r="B51" s="14" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="C51" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="18" customHeight="1">
+      <c r="A52" s="11" t="inlineStr">
+        <is>
+          <t>Hurricane Electric</t>
+        </is>
+      </c>
+      <c r="B52" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="C52" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="18" customHeight="1">
+      <c r="A53" s="13" t="inlineStr">
+        <is>
+          <t>Big River Communications</t>
+        </is>
+      </c>
+      <c r="B53" s="14" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="C53" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="11" t="inlineStr">
+        <is>
+          <t>SiFi Networks</t>
+        </is>
+      </c>
+      <c r="B54" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="C54" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="18" customHeight="1">
+      <c r="A55" s="13" t="inlineStr">
+        <is>
+          <t>MetTel</t>
+        </is>
+      </c>
+      <c r="B55" s="14" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+      <c r="C55" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="18" customHeight="1">
+      <c r="A56" s="11" t="inlineStr">
+        <is>
+          <t>Bell Canada</t>
+        </is>
+      </c>
+      <c r="B56" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="C56" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="18" customHeight="1">
+      <c r="A57" s="13" t="inlineStr">
+        <is>
+          <t>GVTC Communications</t>
+        </is>
+      </c>
+      <c r="B57" s="14" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="C57" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="18" customHeight="1">
+      <c r="A58" s="11" t="inlineStr">
+        <is>
+          <t>Dark Fiber and Infrastructure</t>
+        </is>
+      </c>
+      <c r="B58" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="C58" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="18" customHeight="1">
+      <c r="A59" s="13" t="inlineStr">
+        <is>
+          <t>Sabey Data Centers</t>
+        </is>
+      </c>
+      <c r="B59" s="14" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="C59" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="18" customHeight="1">
+      <c r="A60" s="11" t="inlineStr">
+        <is>
+          <t>Astound Broadband</t>
+        </is>
+      </c>
+      <c r="B60" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="C60" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="18" customHeight="1">
+      <c r="A61" s="13" t="inlineStr">
+        <is>
+          <t>Arvig</t>
+        </is>
+      </c>
+      <c r="B61" s="14" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="C61" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="18" customHeight="1">
+      <c r="A62" s="11" t="inlineStr">
+        <is>
+          <t>EastLink</t>
+        </is>
+      </c>
+      <c r="B62" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="C62" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="18" customHeight="1">
+      <c r="A63" s="13" t="inlineStr">
+        <is>
+          <t>LFT Fiber</t>
+        </is>
+      </c>
+      <c r="B63" s="14" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="C63" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="18" customHeight="1">
+      <c r="A64" s="11" t="inlineStr">
+        <is>
+          <t>Plateau Telecommunications</t>
+        </is>
+      </c>
+      <c r="B64" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="C64" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="18" customHeight="1">
+      <c r="A65" s="13" t="inlineStr">
+        <is>
+          <t>Nitel</t>
+        </is>
+      </c>
+      <c r="B65" s="14" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="C65" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="18" customHeight="1">
+      <c r="A66" s="11" t="inlineStr">
+        <is>
+          <t>ITHAKA</t>
+        </is>
+      </c>
+      <c r="B66" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="C66" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="18" customHeight="1">
+      <c r="A67" s="13" t="inlineStr">
+        <is>
+          <t>Bausch Health</t>
+        </is>
+      </c>
+      <c r="B67" s="14" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="C67" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="18" customHeight="1">
+      <c r="A68" s="11" t="inlineStr">
+        <is>
+          <t>KeyBank</t>
+        </is>
+      </c>
+      <c r="B68" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="C68" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="18" customHeight="1">
+      <c r="A69" s="13" t="inlineStr">
+        <is>
+          <t>BullsEye Telecom</t>
+        </is>
+      </c>
+      <c r="B69" s="14" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="C69" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="18" customHeight="1">
+      <c r="A70" s="11" t="inlineStr">
+        <is>
+          <t>Netceed US</t>
+        </is>
+      </c>
+      <c r="B70" s="12" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="C70" s="12" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="18" customHeight="1">
+      <c r="A71" s="13" t="inlineStr">
+        <is>
+          <t>Lippert</t>
+        </is>
+      </c>
+      <c r="B71" s="14" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="C71" s="14" t="inlineStr">
+        <is>
+          <t>email-queue.json</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
NFL sequences: Gregory Perez, Douglas Neu, Trey Dillen queued; session summary 2026-05-05
</commit_message>
<xml_diff>
--- a/prospects-tracker-new.xlsx
+++ b/prospects-tracker-new.xlsx
@@ -528,7 +528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I405"/>
+  <dimension ref="A1:I409"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -19307,6 +19307,194 @@
       <c r="I405" t="inlineStr">
         <is>
           <t>DoD contractor, Breadcrumb mesh nodes. Cost-reduction focus (27% savings on profile). Park Place/SE merger angle for E2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>Girish Budibetta</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>Global Lead for Data Center Transformation</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>Siemens Energy</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/girish-budibetta-bb52015/</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>Sample-Offer Server (DIMMs), TPM, Optics, DWDM</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>IN_PROGRESS</t>
+        </is>
+      </c>
+      <c r="G406" t="inlineStr">
+        <is>
+          <t>Sequence queued Day 1 2026-05-29</t>
+        </is>
+      </c>
+      <c r="H406" t="inlineStr">
+        <is>
+          <t>2026-05-06</t>
+        </is>
+      </c>
+      <c r="I406" t="inlineStr">
+        <is>
+          <t>19+ yrs DC transformation, AWS partnership expansion, approved vendor</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>Gregory Perez</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>Director of Data Center Operations</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>NFL</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/gregoryperez-nfl</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>Pain-Led TPM (NetApp/Cisco) + Storage</t>
+        </is>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>Active - Sequence Started</t>
+        </is>
+      </c>
+      <c r="G407" t="inlineStr">
+        <is>
+          <t>Sequence queued E1 2026-05-06</t>
+        </is>
+      </c>
+      <c r="H407" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="I407" t="inlineStr">
+        <is>
+          <t>Email: perezg@nfl.com (ZI 98% alt pattern). NFL+Azure AI fresh hook. 6 emails queued.</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>Douglas Neu</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>VP of Technology</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>NFL</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/douglas-neu</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>Sample-Offer Server (DIMMs/Compute) + Optics</t>
+        </is>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>Active - Sequence Started</t>
+        </is>
+      </c>
+      <c r="G408" t="inlineStr">
+        <is>
+          <t>Sequence queued E1 2026-05-12</t>
+        </is>
+      </c>
+      <c r="H408" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="I408" t="inlineStr">
+        <is>
+          <t>Email: douglas.neu@nfl.com (dominant-pattern, no ZI match - monitor for bounce). Kubernetes/compute hook.</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>Trey Dillen</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>Sr. Director of Technology - NFL Films</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>NFL</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/trey-dillen</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>Sample-Offer Network (SFPs/Optics) + DWDM</t>
+        </is>
+      </c>
+      <c r="F409" t="inlineStr">
+        <is>
+          <t>Active - Sequence Started</t>
+        </is>
+      </c>
+      <c r="G409" t="inlineStr">
+        <is>
+          <t>Sequence queued E1 2026-05-18</t>
+        </is>
+      </c>
+      <c r="H409" t="inlineStr">
+        <is>
+          <t>2026-05-05</t>
+        </is>
+      </c>
+      <c r="I409" t="inlineStr">
+        <is>
+          <t>Email: trey.dillen@nfl.com (ZI confirmed). NFL Films 9 intl productions fresh hook. Career trajectory hook.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Major workflow migration: queue to HubSpot AI fields
- CLAUDE.md: added 'bad number on [Name] at [Company]' command to clear call tasks
- osi-outreach-sequence: full rewrite — writes to HubSpot AI fields instead of email-queue.json, new email formatting (no Hi, Best/Andy on all emails including Any thoughts), stagger drives LinkedIn task date not sendDate, LINKED_IN_CONNECT task = enrollment cue
- osi-prospect-qualification: added SEQUENCE line (Network/DWDM/Server/Storage/TPM) as first line of every strategy note
- email-queue.json: 240 contacts migrated to HubSpot AI fields and removed from queue
</commit_message>
<xml_diff>
--- a/prospects-tracker-new.xlsx
+++ b/prospects-tracker-new.xlsx
@@ -597,7 +597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:K248"/>
+  <dimension ref="A2:K264"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -11630,6 +11630,703 @@
       <c r="H248" t="inlineStr">
         <is>
           <t>2026-05-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>Randy Kulman</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>VP, Network Operations &amp; Engineering</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>Dobson Fiber</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/randy-kulman-89375350/</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>Sample-Offer Network (transceivers), DWDM, TPM, Pre-Owned Networking</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="G249" t="inlineStr">
+        <is>
+          <t>6-email sequence queued Day 1 2026-05-28</t>
+        </is>
+      </c>
+      <c r="H249" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="I249" t="inlineStr">
+        <is>
+          <t>Dominant-pattern email rkulman@dobson.net. 12+ fiber builds OK/AR May 2026. 6,500-mile network. ZI credits exhausted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>William Zayas</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Vice President, Network Engineering</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>Dobson Fiber</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/williamzayas/</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>Pain-Led DWDM, Optics Sample, TPM, Pre-Owned Networking</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>6-email sequence queued Day 1 2026-06-03</t>
+        </is>
+      </c>
+      <c r="H250" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="I250" t="inlineStr">
+        <is>
+          <t>Dominant-pattern wzayas@dobson.net. DWDM explicit in headline. 12 new routes OK/AR May 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>Raymond Castor</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>CIO</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>Dobson Fiber</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>rcastor@dobson.net</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>Pain-Led TPM</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="G251" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="H251" t="inlineStr">
+        <is>
+          <t>hubspot-existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>Thomas Claydon</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Sr. Network Systems Engineer</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>Dobson Fiber</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>tclaydon@dobson.net</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>Sample-Offer Network</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="G252" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="H252" t="inlineStr">
+        <is>
+          <t>hubspot-existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>Jason Estridge</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Network Engineer</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>Dobson Fiber</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>jestridge@dobson.net</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>Sample-Offer Network</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="G253" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="H253" t="inlineStr">
+        <is>
+          <t>hubspot-existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>Travis Hedger</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Network Engineer III</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>Dobson Fiber</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>thedger@dobson.net</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>Sample-Offer Network</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="H254" t="inlineStr">
+        <is>
+          <t>hubspot-existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>Evon Williams</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>Optical Network Engineer</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Dobson Fiber</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>ewilliams@dobson.net</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>Sample-Offer Network</t>
+        </is>
+      </c>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="G255" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="H255" t="inlineStr">
+        <is>
+          <t>dominant-pattern</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>William Zayas</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>VP Network Engineering</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>Dobson Fiber</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>wzayas@dobson.net</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>Pain-Led DWDM</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="G256" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="H256" t="inlineStr">
+        <is>
+          <t>hubspot-existing</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>Carl Brown</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Network Engineer</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>Dobson Fiber</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>cbrown@dobson.net</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>Sample-Offer Network</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="G257" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="H257" t="inlineStr">
+        <is>
+          <t>dominant-pattern</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>Danny Abbott</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Network Engineer</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>Dobson Technologies</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>dabbott@dobson.net</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>Sample-Offer Network</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>2026-07-29</t>
+        </is>
+      </c>
+      <c r="G258" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="H258" t="inlineStr">
+        <is>
+          <t>dominant-pattern</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>Joshua Bradley</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Network Engineer</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>Dobson Fiber</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>jbradley@dobson.net</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>Sample-Offer Network</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="G259" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="H259" t="inlineStr">
+        <is>
+          <t>dominant-pattern</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>Jacquie Cossey</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Network Provisioning</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>Dobson Fiber</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>jcossey@dobson.net</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>Sample-Offer Network</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="G260" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="H260" t="inlineStr">
+        <is>
+          <t>dominant-pattern</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>Adam Cavazos</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>VP Network Systems &amp; Engineering</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Dobson Fiber</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>acavazos@dobson.net</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>Pain-Led DWDM</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="G261" t="inlineStr">
+        <is>
+          <t>2026-05-27</t>
+        </is>
+      </c>
+      <c r="H261" t="inlineStr">
+        <is>
+          <t>dominant-pattern</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>Andy Hulscher</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Chief Operations Officer</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>Alliance Communications</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/andy-hulscher-04886b6/</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>Sample-Offer Network</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>Sequence Active</t>
+        </is>
+      </c>
+      <c r="G262" t="inlineStr">
+        <is>
+          <t>Email sequence queued Day 1 2026-05-29</t>
+        </is>
+      </c>
+      <c r="H262" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>dominant-pattern email andyh@alliance.coop | CFO retired May 8 2026 after 30 yrs + Luverne MN fiber expansion</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>Derek Ridgway</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Network Administrator</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>Alliance Communications</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/derek-ridgway-676ba2148/</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>Sample-Offer Network</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>Sequence Active</t>
+        </is>
+      </c>
+      <c r="G263" t="inlineStr">
+        <is>
+          <t>Email sequence queued Day 1 2026-06-04</t>
+        </is>
+      </c>
+      <c r="H263" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="I263" t="inlineStr">
+        <is>
+          <t>verified-pattern email derekr@alliance.coop (ZI FULL_MATCH score 94) | CFO retired May 8 2026 + Luverne MN expansion</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>Darin Egenes</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>Systems Administrator</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>Alliance Communications</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/darin-egenes-7180842/</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>Sample-Offer Server</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>Sequence Active</t>
+        </is>
+      </c>
+      <c r="G264" t="inlineStr">
+        <is>
+          <t>Email sequence queued Day 1 2026-06-10</t>
+        </is>
+      </c>
+      <c r="H264" t="inlineStr">
+        <is>
+          <t>2026-05-28</t>
+        </is>
+      </c>
+      <c r="I264" t="inlineStr">
+        <is>
+          <t>dominant-pattern email darine@alliance.coop | Path A verified LinkedIn | remote Seattle WA | CFO retired May 8 2026 + Luverne MN expansion</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Index Exchange company mode: 7 sequenced, ZI web-app fallback rule added to qualification skill, session notes + test prompt
</commit_message>
<xml_diff>
--- a/prospects-tracker-new.xlsx
+++ b/prospects-tracker-new.xlsx
@@ -597,7 +597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:K264"/>
+  <dimension ref="A2:K271"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="2">
@@ -12327,6 +12327,335 @@
       <c r="I264" t="inlineStr">
         <is>
           <t>dominant-pattern email darine@alliance.coop | Path A verified LinkedIn | remote Seattle WA | CFO retired May 8 2026 + Luverne MN expansion</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>Friedrich Seifts</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Vice President: Technology Operations</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>Index Exchange</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/fseifts/</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>Sample-Offer Server (DIMM), TPM + optics follow</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>Contact created 226189354417</t>
+        </is>
+      </c>
+      <c r="G265" t="inlineStr">
+        <is>
+          <t>Sequence drafted to AI fields, enroll Day 1 2026-06-04</t>
+        </is>
+      </c>
+      <c r="H265" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="I265" t="inlineStr">
+        <is>
+          <t>Hook: MLB/Disney Streaming infra builder; Index Cloud buildout Apr 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>Michael O'Dea</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Director of System Operations</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>Index Exchange</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/modea/</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>Sample-Offer Server (DIMM), TPM + storage follow</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>Contact created 226188750943</t>
+        </is>
+      </c>
+      <c r="G266" t="inlineStr">
+        <is>
+          <t>Sequence drafted to AI fields, enroll Day 1 2026-06-10</t>
+        </is>
+      </c>
+      <c r="H266" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="I266" t="inlineStr">
+        <is>
+          <t>Hook: joined Apr 2026 from Disney Streaming (7 yrs infra); ex MLBAM/BAMTech</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>Tony Savor</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>VP, Platform Engineering</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>Index Exchange</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/tony-savor-7869271/</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>Sample-Offer Server (DIMM), optics + TPM + storage follow</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>Contact created 226189889046</t>
+        </is>
+      </c>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>Sequence drafted to AI fields, enroll Day 1 2026-06-16</t>
+        </is>
+      </c>
+      <c r="H267" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="I267" t="inlineStr">
+        <is>
+          <t>Hook: ex Google GKE + Facebook storage infra; planet scale efficiency posts; U of T on prem research</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>Bo Blanton</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Director, Data Systems</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>Index Exchange</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/wyndham/</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>Sample-Offer Server (DIMM), storage + TPM follow</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>Contact created 226186213420</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>Sequence drafted to AI fields, enroll Day 1 2026-06-22</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="I268" t="inlineStr">
+        <is>
+          <t>Hook: Berkeley chem PhD to petabyte data systems; ex ASAPP with Seifts</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>Luis Alfredo Morales Lora</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Engineering Lead Manager - Network Engineering</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>Index Exchange</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/luis-alfredo-morales-lora-182ba684/</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>Sample-Offer Network (SFP), DWDM + pre-owned + TPM follow</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>Contact created 226186662295</t>
+        </is>
+      </c>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>Sequence drafted to AI fields, enroll Day 1 2026-06-26</t>
+        </is>
+      </c>
+      <c r="H269" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="I269" t="inlineStr">
+        <is>
+          <t>Hook: CCIE 47341 RS|SP; AlticeDo ISP backbone to Cisco to IX network engineering lead</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>Joshua Hoblitt</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>Staff Storage Engineer</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>Index Exchange</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/jhoblitt/</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>Sample-Offer Server (DIMM), storage + TPM follow</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>Contact created 226207041068</t>
+        </is>
+      </c>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>Sequence drafted to AI fields, enroll Day 1 2026-07-13</t>
+        </is>
+      </c>
+      <c r="H270" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="I270" t="inlineStr">
+        <is>
+          <t>Hook: joined ~Feb 2026; shared Rook v1.19.5 Ceph release last month</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>Edward Alvarez</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Staff Network Engineer</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>Index Exchange</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/in/edward-alvarez-9893573b/</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>Sample-Offer Network (SFP), pre-owned + DWDM + TPM follow</t>
+        </is>
+      </c>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>Contact created 226206123378</t>
+        </is>
+      </c>
+      <c r="G271" t="inlineStr">
+        <is>
+          <t>Sequence drafted to AI fields, enroll Day 1 2026-07-17</t>
+        </is>
+      </c>
+      <c r="H271" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+      <c r="I271" t="inlineStr">
+        <is>
+          <t>Hook: AlticeDo to SIG to IX network; RIT MS; same lineage as manager Luis</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update obsidian-vault skill: new OSI-Notes vault path, direct API calls; add nightly vault backup task
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/prospects-tracker-new.xlsx
+++ b/prospects-tracker-new.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mini\Documents\osi-claude-brain\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\osi-claude-brain\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A1F7FB2-A4C6-4334-A53C-05474D7CCCF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D17ED24D-B2D6-4E86-A685-F07F8EE733E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="7665" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="37215" yWindow="7935" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tab1" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="65">
   <si>
     <t>Name</t>
   </si>
@@ -179,6 +179,48 @@
   </si>
   <si>
     <t>No email found. LinkedIn InMail path. Server Engineer at SBG -- DIMMs wedge for 6-ISP compute standardization.</t>
+  </si>
+  <si>
+    <t>Joe Brannan</t>
+  </si>
+  <si>
+    <t>VP Core Infrastructure Services</t>
+  </si>
+  <si>
+    <t>Lincoln Financial Group</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/joe-brannan-6828634/</t>
+  </si>
+  <si>
+    <t>Pain-Led TPM (DIMMs, pre-owned Cisco, optics secondary)</t>
+  </si>
+  <si>
+    <t>Sequenced</t>
+  </si>
+  <si>
+    <t>Enroll in HubSpot sequence 2026-06-12</t>
+  </si>
+  <si>
+    <t>joe.brannan@lfg.com | direct +1 (336) 860-5805 | mobile +1 (336) 681-4949 | HubSpot ID 227841622697</t>
+  </si>
+  <si>
+    <t>Dan Vetro</t>
+  </si>
+  <si>
+    <t>VP Infrastructure, UCC, Network and Contact Center</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/danvetro/</t>
+  </si>
+  <si>
+    <t>Pain-Led TPM (optics, pre-owned Cisco, DIMMs secondary)</t>
+  </si>
+  <si>
+    <t>Enroll in HubSpot sequence 2026-06-18</t>
+  </si>
+  <si>
+    <t>dan.vetro@lfg.com | no phone (ZI no record) | HubSpot ID 227837492758 | email: dominant-pattern</t>
   </si>
 </sst>
 </file>
@@ -533,7 +575,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -680,6 +722,64 @@
       </c>
       <c r="I5" t="s">
         <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D6" t="s">
+        <v>54</v>
+      </c>
+      <c r="E6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F6" t="s">
+        <v>56</v>
+      </c>
+      <c r="G6" t="s">
+        <v>57</v>
+      </c>
+      <c r="H6" s="2">
+        <v>46184</v>
+      </c>
+      <c r="I6" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>59</v>
+      </c>
+      <c r="B7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C7" t="s">
+        <v>53</v>
+      </c>
+      <c r="D7" t="s">
+        <v>61</v>
+      </c>
+      <c r="E7" t="s">
+        <v>62</v>
+      </c>
+      <c r="F7" t="s">
+        <v>56</v>
+      </c>
+      <c r="G7" t="s">
+        <v>63</v>
+      </c>
+      <c r="H7" s="2">
+        <v>46184</v>
+      </c>
+      <c r="I7" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>